<commit_message>
Batch Edit page, UI improvements, and function updates
</commit_message>
<xml_diff>
--- a/Taxonomy/taxonomy_source.xlsx
+++ b/Taxonomy/taxonomy_source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nzies-my.sharepoint.com/personal/felix_zareievaux_earthsciences_nz/Documents/Documents/R Apps/Backups/Aurora-GitHub-2-2026.04.15/Taxonomy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nzies-my.sharepoint.com/personal/felix_zareievaux_earthsciences_nz/Documents/Documents/R Apps/Backups/Aurora-2026.08.21-git/Taxonomy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{3559198D-1609-48EA-B65B-98F53267ECCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56E2A2DB-DABE-4CC8-AD44-6349AC005188}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{3559198D-1609-48EA-B65B-98F53267ECCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E8956C1-5BBB-4573-86B2-478BA1BE8C2F}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="960" windowWidth="29040" windowHeight="15720" xr2:uid="{56C7A9C3-D804-4863-AB3B-C9D918D26E1A}"/>
+    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" xr2:uid="{56C7A9C3-D804-4863-AB3B-C9D918D26E1A}"/>
   </bookViews>
   <sheets>
     <sheet name="source" sheetId="4" r:id="rId1"/>

</xml_diff>